<commit_message>
added team names and members
</commit_message>
<xml_diff>
--- a/teams-and-rosters/CS320-Sp25-102-roster.xlsx
+++ b/teams-and-rosters/CS320-Sp25-102-roster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\teams-and-rosters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA5255D-9E34-4690-A305-8EBF35327913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71B946B-E927-4F63-8B7A-57090B62F2DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="315" yWindow="1050" windowWidth="12720" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="645" yWindow="615" windowWidth="22050" windowHeight="14730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cs320-102-sp25-roster" sheetId="1" r:id="rId1"/>
@@ -94,9 +94,6 @@
     <t>Onyejesi</t>
   </si>
   <si>
-    <t>Chibudom</t>
-  </si>
-  <si>
     <t>Reppert</t>
   </si>
   <si>
@@ -134,6 +131,9 @@
   </si>
   <si>
     <t>CybMgt</t>
+  </si>
+  <si>
+    <t>Ethan</t>
   </si>
 </sst>
 </file>
@@ -1159,10 +1159,10 @@
     </row>
     <row r="3" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>6</v>
@@ -1179,7 +1179,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>10</v>
@@ -1260,7 +1260,7 @@
         <v>23</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>6</v>
@@ -1271,10 +1271,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>16</v>
@@ -1285,10 +1285,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>6</v>
@@ -1299,10 +1299,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>22</v>
@@ -1313,10 +1313,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>6</v>
@@ -1327,10 +1327,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>22</v>

</xml_diff>